<commit_message>
Refocus Scenario 2 basket on Asian AI hardware
Replace the platform and conglomerate names (Sony, Hitachi, SoftBank,
Keyence, Tencent, Alibaba, Xiaomi) with AI-hardware suppliers (Disco,
Shin-Etsu, ASE, Ibiden, Hon Hai, Quanta, Delta). Raise basket vol
regimes to 27%/50% and raw-basket implied vol to 33% for the more
concentrated semiconductor basket, re-run pricing, and update the deck,
Excel model, backtest tickers and strategy write-up.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAuaaaJzDmbMdV7YcMwaXR
</commit_message>
<xml_diff>
--- a/pricing/Asia-Digital-Bridge-Pricer.xlsx
+++ b/pricing/Asia-Digital-Bridge-Pricer.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pricer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Payoff" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Design Dial" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MC Results" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Risk" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Basket" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Term Sheet" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Payoff" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design Dial" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MC Results" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basket" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Term Sheet" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>0.9571179294083131</v>
+        <v>0.9607321121415533</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -1460,7 +1460,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Placeholder market inputs (regime vol 22%/45%, OIS 3.75%, raw-basket implied vol 30%). Forward simulation, NOT a historical backtest.</t>
+          <t>Placeholder market inputs (regime vol 27%/50%, OIS 3.75%, raw-basket implied vol 33%). Forward simulation, NOT a historical backtest.</t>
         </is>
       </c>
     </row>
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.1853540108796246</v>
+        <v>0.1860539280424679</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1.639343270583038</v>
+        <v>1.63317621728325</v>
       </c>
     </row>
     <row r="7">
@@ -1508,10 +1508,10 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>0.1735523064897174</v>
+        <v>0.1741799269314789</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>1.75082000669977</v>
+        <v>1.744511297967323</v>
       </c>
     </row>
     <row r="8">
@@ -1521,10 +1521,10 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0.1954112042026089</v>
+        <v>0.1960663542864369</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>1.554971485135707</v>
+        <v>1.549775592640309</v>
       </c>
     </row>
     <row r="9">
@@ -1534,10 +1534,10 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.1818706486654591</v>
+        <v>0.1824276751997126</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>1.670741555279868</v>
+        <v>1.665640095881496</v>
       </c>
     </row>
     <row r="11">
@@ -1586,19 +1586,19 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>3.530515235837419</v>
+        <v>3.512186083785713</v>
       </c>
       <c r="C13" s="21" t="n">
-        <v>1.046351017763377</v>
+        <v>1.000788433124645</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0.4826</v>
+        <v>0.4993</v>
       </c>
       <c r="E13" s="21" t="n">
-        <v>1.438270526941504</v>
+        <v>1.313567175584545</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.3539</v>
+        <v>0.3956</v>
       </c>
     </row>
     <row r="14">
@@ -1608,19 +1608,19 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>2.150055231259482</v>
+        <v>2.140670419519987</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>1.35953399966631</v>
+        <v>1.331406726874817</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0.2775</v>
+        <v>0.2902</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>1.586706176934527</v>
+        <v>1.513663487801304</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.1766</v>
+        <v>0.2043</v>
       </c>
     </row>
     <row r="15">
@@ -1630,19 +1630,19 @@
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>1.606418622737814</v>
+        <v>1.60015327453743</v>
       </c>
       <c r="C15" s="21" t="n">
-        <v>1.404570298256958</v>
+        <v>1.381701838554376</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>0.1934</v>
+        <v>0.2056</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>1.586600811829943</v>
+        <v>1.527810396317611</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.1163</v>
+        <v>0.1383</v>
       </c>
     </row>
     <row r="16">
@@ -1652,19 +1652,19 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>1.238211784679967</v>
+        <v>1.233937568841018</v>
       </c>
       <c r="C16" s="21" t="n">
-        <v>1.424215265462836</v>
+        <v>1.405143381388603</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0.1302</v>
+        <v>0.1385</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>1.574688456874342</v>
+        <v>1.525976582332643</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.0727</v>
+        <v>0.0873</v>
       </c>
     </row>
     <row r="17">
@@ -1674,19 +1674,19 @@
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>0.9528576109123992</v>
+        <v>0.8871088063348338</v>
       </c>
       <c r="C17" s="21" t="n">
-        <v>1.209820298217498</v>
+        <v>1.100287601936849</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0.3826</v>
+        <v>0.4506</v>
       </c>
       <c r="E17" s="21" t="n">
-        <v>1.481512616377541</v>
+        <v>1.331020479030028</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.2655</v>
+        <v>0.3448</v>
       </c>
     </row>
     <row r="19">
@@ -1745,25 +1745,25 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>1.374774154686243</v>
+        <v>1.378856868087378</v>
       </c>
       <c r="C21" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="21" t="n">
-        <v>1.236751647441378</v>
+        <v>1.244587127782382</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>2.250880860761919</v>
+        <v>2.250585868677348</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>0.03082089667991017</v>
+        <v>0.03175134464910978</v>
       </c>
       <c r="G21" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>0.3032</v>
+        <v>0.29715</v>
       </c>
     </row>
     <row r="22">
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>1.403964275414697</v>
+        <v>1.422897028518891</v>
       </c>
       <c r="C22" s="21" t="n">
         <v>1</v>
@@ -1782,7 +1782,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>2.864640120476828</v>
+        <v>3.071916081299568</v>
       </c>
       <c r="F22" s="7" t="n">
         <v>0</v>
@@ -1791,7 +1791,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>0.5116000000000001</v>
+        <v>0.5573</v>
       </c>
     </row>
     <row r="23">
@@ -1801,25 +1801,25 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>1.231966993727667</v>
+        <v>1.233184420604062</v>
       </c>
       <c r="C23" s="21" t="n">
-        <v>0.3220723113824985</v>
+        <v>0.2370151633968244</v>
       </c>
       <c r="D23" s="21" t="n">
-        <v>0.980988041886751</v>
+        <v>0.8921854637891187</v>
       </c>
       <c r="E23" s="21" t="n">
-        <v>2.956892718410845</v>
+        <v>3.335582812958274</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>-0.002738387987202329</v>
+        <v>-0.01616523847580398</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>0.5116000000000001</v>
+        <v>0.5572</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>0.5116000000000001</v>
+        <v>0.5573</v>
       </c>
     </row>
     <row r="24">
@@ -1829,25 +1829,25 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>1.519610813141407</v>
+        <v>1.496605471555177</v>
       </c>
       <c r="C24" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>1.406357251024726</v>
+        <v>1.382398322640645</v>
       </c>
       <c r="E24" s="21" t="n">
-        <v>2.507310452483311</v>
+        <v>2.463509535225619</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>0.04992075830692633</v>
+        <v>0.04734667158213113</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>0.19605</v>
+        <v>0.2073</v>
       </c>
     </row>
     <row r="25">
@@ -1857,25 +1857,25 @@
         </is>
       </c>
       <c r="B25" s="21" t="n">
-        <v>1.620415621724595</v>
+        <v>1.623864149006904</v>
       </c>
       <c r="C25" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="21" t="n">
-        <v>1.200312989889312</v>
+        <v>1.08930491715661</v>
       </c>
       <c r="E25" s="21" t="n">
-        <v>3.523027524280381</v>
+        <v>3.7633752764057</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>0.02642633586804644</v>
+        <v>0.01229494062704617</v>
       </c>
       <c r="G25" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>0.3874</v>
+        <v>0.4542</v>
       </c>
     </row>
     <row r="26">
@@ -1885,25 +1885,25 @@
         </is>
       </c>
       <c r="B26" s="21" t="n">
-        <v>1.51985065075269</v>
+        <v>1.5213525635797</v>
       </c>
       <c r="C26" s="21" t="n">
-        <v>0.3973335442721443</v>
+        <v>0.2924004069597267</v>
       </c>
       <c r="D26" s="21" t="n">
-        <v>1.210223424355612</v>
+        <v>1.100669632088966</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>3.647853672349304</v>
+        <v>4.115035333515426</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>0.02763274963638052</v>
+        <v>0.01379699067368456</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>0.38715</v>
+        <v>0.45405</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>0.3874</v>
+        <v>0.4542</v>
       </c>
     </row>
     <row r="27">
@@ -1913,25 +1913,25 @@
         </is>
       </c>
       <c r="B27" s="21" t="n">
-        <v>1.690944561447927</v>
+        <v>1.632414751970672</v>
       </c>
       <c r="C27" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>1.590809045802867</v>
+        <v>1.531600858896554</v>
       </c>
       <c r="E27" s="21" t="n">
-        <v>2.78912868848549</v>
+        <v>2.688998865486607</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>0.06856901965108109</v>
+        <v>0.06279467947640494</v>
       </c>
       <c r="G27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.11955</v>
+        <v>0.1406</v>
       </c>
     </row>
     <row r="28">
@@ -1941,25 +1941,25 @@
         </is>
       </c>
       <c r="B28" s="21" t="n">
-        <v>1.914015543752787</v>
+        <v>1.893299408673269</v>
       </c>
       <c r="C28" s="21" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>1.469783658683808</v>
+        <v>1.317471381777234</v>
       </c>
       <c r="E28" s="21" t="n">
-        <v>4.335265619304733</v>
+        <v>4.616413314763465</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>0.05655800526845123</v>
+        <v>0.04017373720036987</v>
       </c>
       <c r="G28" s="8" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>0.27515</v>
+        <v>0.35185</v>
       </c>
     </row>
     <row r="29">
@@ -1969,31 +1969,31 @@
         </is>
       </c>
       <c r="B29" s="21" t="n">
-        <v>1.875006402244573</v>
+        <v>1.876859279147221</v>
       </c>
       <c r="C29" s="21" t="n">
-        <v>0.4901816760533972</v>
+        <v>0.3607279667886384</v>
       </c>
       <c r="D29" s="21" t="n">
-        <v>1.493026086273238</v>
+        <v>1.357871976368822</v>
       </c>
       <c r="E29" s="21" t="n">
-        <v>4.500277041509994</v>
+        <v>5.076628806904743</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>0.05892882610192751</v>
+        <v>0.04467170554813005</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>0.2751</v>
+        <v>0.35175</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>0.27515</v>
+        <v>0.35185</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>7Y UST proxy multiple: 1.38x. Mean VT exposure 41%; realised index vol 9.8%.</t>
+          <t>7Y UST proxy multiple: 1.38x. Mean VT exposure 34%; realised index vol 9.8%.</t>
         </is>
       </c>
     </row>
@@ -2132,17 +2132,17 @@
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>Asia tech crash: basket -30% in 1M, vol 22-&gt;45%, rates -50bp</t>
+          <t>AI hardware crash: basket -30% in 1M, vol 27%-&gt;50%, rates -50bp</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>0.884090909090909</v>
+        <v>0.9055555555555556</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>-0.005</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.8556997659849921</v>
+        <v>0.8751914881799825</v>
       </c>
       <c r="E11" s="16">
         <f>(D11-$B$3)*Pricer!$B$5</f>
@@ -2160,13 +2160,13 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.9259259259259259</v>
       </c>
       <c r="C12" s="7" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.8800642195046026</v>
+        <v>0.8973891837882668</v>
       </c>
       <c r="E12" s="16">
         <f>(D12-$B$3)*Pricer!$B$5</f>
@@ -2184,13 +2184,13 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>0.9318181818181818</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>0.01</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>0.9156691649609003</v>
+        <v>0.930656522185227</v>
       </c>
       <c r="E13" s="16">
         <f>(D13-$B$3)*Pricer!$B$5</f>
@@ -2208,13 +2208,13 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>1.113636363636364</v>
+        <v>1.092592592592593</v>
       </c>
       <c r="C14" s="7" t="n">
         <v>-0.005</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>1.109538475486936</v>
+        <v>1.082940789753381</v>
       </c>
       <c r="E14" s="16">
         <f>(D14-$B$3)*Pricer!$B$5</f>
@@ -2311,7 +2311,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Underlying basket: Asian digital-transformation leaders (equal weight, USD quanto)</t>
+          <t>Underlying basket: Asian AI-hardware leaders (equal weight, USD quanto)</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Foundry / AI compute</t>
+          <t>Foundry / AI accelerators</t>
         </is>
       </c>
       <c r="E5" s="24">
@@ -2403,22 +2403,22 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>005930 KS</t>
+          <t>2454 TT</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Samsung Electronics</t>
+          <t>MediaTek</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>Memory / devices</t>
+          <t>Custom AI ASICs / edge AI</t>
         </is>
       </c>
       <c r="E6" s="24">
@@ -2467,22 +2467,22 @@
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>2454 TT</t>
+          <t>005930 KS</t>
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>MediaTek</t>
+          <t>Samsung Electronics</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>Edge-AI chips</t>
+          <t>HBM / memory</t>
         </is>
       </c>
       <c r="E8" s="24">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Chip equipment</t>
+          <t>Wafer-fab equipment</t>
         </is>
       </c>
       <c r="E9" s="24">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>Chip testing</t>
+          <t>AI chip testing</t>
         </is>
       </c>
       <c r="E10" s="24">
@@ -2563,12 +2563,12 @@
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>6758 JT</t>
+          <t>6146 JT</t>
         </is>
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>Sony Group</t>
+          <t>Disco</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>Bridge: sensors, content</t>
+          <t>Dicing / grinding for HBM</t>
         </is>
       </c>
       <c r="E11" s="24">
@@ -2595,12 +2595,12 @@
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>6501 JT</t>
+          <t>4063 JT</t>
         </is>
       </c>
       <c r="B12" s="23" t="inlineStr">
         <is>
-          <t>Hitachi</t>
+          <t>Shin-Etsu Chemical</t>
         </is>
       </c>
       <c r="C12" s="23" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>Bridge: industrial digital</t>
+          <t>Silicon wafers / materials</t>
         </is>
       </c>
       <c r="E12" s="24">
@@ -2627,22 +2627,22 @@
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>9984 JT</t>
+          <t>3711 TT</t>
         </is>
       </c>
       <c r="B13" s="23" t="inlineStr">
         <is>
-          <t>SoftBank Group</t>
+          <t>ASE Technology</t>
         </is>
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>Bridge: AI investing</t>
+          <t>Advanced packaging</t>
         </is>
       </c>
       <c r="E13" s="24">
@@ -2659,12 +2659,12 @@
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>6861 JT</t>
+          <t>4062 JT</t>
         </is>
       </c>
       <c r="B14" s="23" t="inlineStr">
         <is>
-          <t>Keyence</t>
+          <t>Ibiden</t>
         </is>
       </c>
       <c r="C14" s="23" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>Factory automation</t>
+          <t>AI chip substrates</t>
         </is>
       </c>
       <c r="E14" s="24">
@@ -2691,22 +2691,22 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>700 HK</t>
+          <t>2317 TT</t>
         </is>
       </c>
       <c r="B15" s="23" t="inlineStr">
         <is>
-          <t>Tencent</t>
+          <t>Hon Hai (Foxconn)</t>
         </is>
       </c>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>HK/CN</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="D15" s="23" t="inlineStr">
         <is>
-          <t>Platforms / cloud</t>
+          <t>AI server assembly</t>
         </is>
       </c>
       <c r="E15" s="24">
@@ -2723,22 +2723,22 @@
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
         <is>
-          <t>9988 HK</t>
+          <t>2382 TT</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Alibaba</t>
+          <t>Quanta Computer</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>HK/CN</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Cloud / AI models</t>
+          <t>AI servers</t>
         </is>
       </c>
       <c r="E16" s="24">
@@ -2755,22 +2755,22 @@
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
         <is>
-          <t>1810 HK</t>
+          <t>2308 TT</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Xiaomi</t>
+          <t>Delta Electronics</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>HK/CN</t>
+          <t>TW</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Devices / EV / IoT</t>
+          <t>Data-centre power / cooling</t>
         </is>
       </c>
       <c r="E17" s="24">
@@ -2798,7 +2798,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Excluded on purpose: renewables, real estate, data-centre REITs (overlap with family businesses); names on US restriction lists (e.g. SMIC, Hikvision). Rules: market cap &gt;= USD 250M; listed ADV &gt; USD 5M over 6M; no OFAC-sanctioned countries; Bloomberg searchable.</t>
+          <t>Excluded on purpose: data-centre operators/REITs, telecom towers, renewables, real estate (overlap with family businesses); names on US restriction lists (e.g. SMIC). Rules: market cap &gt;= USD 250M; listed ADV &gt; USD 5M over 6M; no OFAC-sanctioned countries; Bloomberg searchable.</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>Natixis Asia Digital Bridge 10% VT Index (USD, 1% decrement), on an equal-weight 13-stock basket</t>
+          <t>Natixis Asia Digital Bridge 10% VT Index (USD, 1% decrement), on an equal-weight basket of 13 Asian AI-hardware stocks</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch Scenario 2 to a 60/40 barbell: growth note + 10% Phoenix
Add pricing/scenario2_barbell.py: one-factor two-regime model shared by
the Phoenix pricer and a joint 7Y portfolio simulation. Phoenix: 5Y USD
autocall on an equal-weight TSMC / SK Hynix / Tokyo Electron basket,
10% p.a. conditional quarterly coupon with memory, 50% European barrier.
Add Phoenix and Barbell tabs to the Excel pricer, rebuild the deck as
deck/Asia-AI-Hardware-Barbell.pptx with the corrected outlook draft, and
document the barbell in the strategy write-up.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAuaaaJzDmbMdV7YcMwaXR
</commit_message>
<xml_diff>
--- a/pricing/Asia-Digital-Bridge-Pricer.xlsx
+++ b/pricing/Asia-Digital-Bridge-Pricer.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basket" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Term Sheet" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phoenix" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Barbell" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -59,6 +61,10 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00008000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
     <font>
@@ -68,10 +74,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00008000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -109,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,34 +120,38 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -230,7 +236,7 @@
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
       <text>
-        <t>Client mandate: USD 100Mn (rules, Scenario 2)</t>
+        <t>Growth sleeve = total mandate x growth allocation (Barbell tab)</t>
       </text>
     </comment>
     <comment ref="B6" authorId="0" shapeId="0">
@@ -281,6 +287,21 @@
     <comment ref="B9" authorId="0" shapeId="0">
       <text>
         <t>Rules: combined net worth exceeding USD 2Bn</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Team</author>
+  </authors>
+  <commentList>
+    <comment ref="B4" authorId="0" shapeId="0">
+      <text>
+        <t>Rules: USD 100Mn</t>
       </text>
     </comment>
   </commentList>
@@ -576,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -630,8 +651,9 @@
           <t>Notional (USD)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>100000000</v>
+      <c r="B5" s="5">
+        <f>Barbell!B4*Barbell!B5</f>
+        <v/>
       </c>
       <c r="D5" s="6" t="n">
         <v>1</v>
@@ -942,6 +964,37 @@
         <v/>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Lock + averaging option cost / base option cost (MC)</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>0.980509667917747</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>From scenario2_vt_note.py feature menu (same paths)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>PARTICIPATION WITH LEGACY LOCK + 12M AVERAGING</t>
+        </is>
+      </c>
+      <c r="B29" s="15">
+        <f>IF(B21*B28&gt;0,B17/(B21*B28),0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Proposed product terms</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -985,7 +1038,7 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B3" s="18">
+      <c r="B3" s="19">
         <f>Pricer!B23</f>
         <v/>
       </c>
@@ -994,7 +1047,7 @@
           <t>Protection</t>
         </is>
       </c>
-      <c r="D3" s="18">
+      <c r="D3" s="19">
         <f>Pricer!B7</f>
         <v/>
       </c>
@@ -1005,7 +1058,7 @@
           <t>Tenor (years)</t>
         </is>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="20">
         <f>Pricer!B6</f>
         <v/>
       </c>
@@ -1310,19 +1363,19 @@
           <t>Target vol \ decrement</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="20" t="n">
+      <c r="C4" s="21" t="n">
         <v>0.01</v>
       </c>
-      <c r="D4" s="20" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.02</v>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E4" s="21" t="n">
         <v>0.03</v>
       </c>
-      <c r="F4" s="20" t="n">
+      <c r="F4" s="21" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -1588,13 +1641,13 @@
       <c r="B13" s="8" t="n">
         <v>3.512186083785713</v>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C13" s="22" t="n">
         <v>1.000788433124645</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>0.4993</v>
       </c>
-      <c r="E13" s="21" t="n">
+      <c r="E13" s="22" t="n">
         <v>1.313567175584545</v>
       </c>
       <c r="F13" s="8" t="n">
@@ -1610,13 +1663,13 @@
       <c r="B14" s="8" t="n">
         <v>2.140670419519987</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="22" t="n">
         <v>1.331406726874817</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2902</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="22" t="n">
         <v>1.513663487801304</v>
       </c>
       <c r="F14" s="8" t="n">
@@ -1632,13 +1685,13 @@
       <c r="B15" s="8" t="n">
         <v>1.60015327453743</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="22" t="n">
         <v>1.381701838554376</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>0.2056</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="22" t="n">
         <v>1.527810396317611</v>
       </c>
       <c r="F15" s="8" t="n">
@@ -1654,13 +1707,13 @@
       <c r="B16" s="8" t="n">
         <v>1.233937568841018</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="22" t="n">
         <v>1.405143381388603</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>0.1385</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="22" t="n">
         <v>1.525976582332643</v>
       </c>
       <c r="F16" s="8" t="n">
@@ -1676,13 +1729,13 @@
       <c r="B17" s="8" t="n">
         <v>0.8871088063348338</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="22" t="n">
         <v>1.100287601936849</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>0.4506</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="22" t="n">
         <v>1.331020479030028</v>
       </c>
       <c r="F17" s="8" t="n">
@@ -1744,16 +1797,16 @@
           <t>3% p.a. | VT note</t>
         </is>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="22" t="n">
         <v>1.378856868087378</v>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="22" t="n">
         <v>1.244587127782382</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="22" t="n">
         <v>2.250585868677348</v>
       </c>
       <c r="F21" s="7" t="n">
@@ -1772,16 +1825,16 @@
           <t>3% p.a. | Protected note on raw basket</t>
         </is>
       </c>
-      <c r="B22" s="21" t="n">
+      <c r="B22" s="22" t="n">
         <v>1.422897028518891</v>
       </c>
-      <c r="C22" s="21" t="n">
+      <c r="C22" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="21" t="n">
+      <c r="D22" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="21" t="n">
+      <c r="E22" s="22" t="n">
         <v>3.071916081299568</v>
       </c>
       <c r="F22" s="7" t="n">
@@ -1800,16 +1853,16 @@
           <t>3% p.a. | Direct basket</t>
         </is>
       </c>
-      <c r="B23" s="21" t="n">
+      <c r="B23" s="22" t="n">
         <v>1.233184420604062</v>
       </c>
-      <c r="C23" s="21" t="n">
+      <c r="C23" s="22" t="n">
         <v>0.2370151633968244</v>
       </c>
-      <c r="D23" s="21" t="n">
+      <c r="D23" s="22" t="n">
         <v>0.8921854637891187</v>
       </c>
-      <c r="E23" s="21" t="n">
+      <c r="E23" s="22" t="n">
         <v>3.335582812958274</v>
       </c>
       <c r="F23" s="7" t="n">
@@ -1828,16 +1881,16 @@
           <t>6% p.a. | VT note</t>
         </is>
       </c>
-      <c r="B24" s="21" t="n">
+      <c r="B24" s="22" t="n">
         <v>1.496605471555177</v>
       </c>
-      <c r="C24" s="21" t="n">
+      <c r="C24" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="21" t="n">
+      <c r="D24" s="22" t="n">
         <v>1.382398322640645</v>
       </c>
-      <c r="E24" s="21" t="n">
+      <c r="E24" s="22" t="n">
         <v>2.463509535225619</v>
       </c>
       <c r="F24" s="7" t="n">
@@ -1856,16 +1909,16 @@
           <t>6% p.a. | Protected note on raw basket</t>
         </is>
       </c>
-      <c r="B25" s="21" t="n">
+      <c r="B25" s="22" t="n">
         <v>1.623864149006904</v>
       </c>
-      <c r="C25" s="21" t="n">
+      <c r="C25" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="21" t="n">
+      <c r="D25" s="22" t="n">
         <v>1.08930491715661</v>
       </c>
-      <c r="E25" s="21" t="n">
+      <c r="E25" s="22" t="n">
         <v>3.7633752764057</v>
       </c>
       <c r="F25" s="7" t="n">
@@ -1884,16 +1937,16 @@
           <t>6% p.a. | Direct basket</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n">
+      <c r="B26" s="22" t="n">
         <v>1.5213525635797</v>
       </c>
-      <c r="C26" s="21" t="n">
+      <c r="C26" s="22" t="n">
         <v>0.2924004069597267</v>
       </c>
-      <c r="D26" s="21" t="n">
+      <c r="D26" s="22" t="n">
         <v>1.100669632088966</v>
       </c>
-      <c r="E26" s="21" t="n">
+      <c r="E26" s="22" t="n">
         <v>4.115035333515426</v>
       </c>
       <c r="F26" s="7" t="n">
@@ -1912,16 +1965,16 @@
           <t>9% p.a. | VT note</t>
         </is>
       </c>
-      <c r="B27" s="21" t="n">
+      <c r="B27" s="22" t="n">
         <v>1.632414751970672</v>
       </c>
-      <c r="C27" s="21" t="n">
+      <c r="C27" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="21" t="n">
+      <c r="D27" s="22" t="n">
         <v>1.531600858896554</v>
       </c>
-      <c r="E27" s="21" t="n">
+      <c r="E27" s="22" t="n">
         <v>2.688998865486607</v>
       </c>
       <c r="F27" s="7" t="n">
@@ -1940,16 +1993,16 @@
           <t>9% p.a. | Protected note on raw basket</t>
         </is>
       </c>
-      <c r="B28" s="21" t="n">
+      <c r="B28" s="22" t="n">
         <v>1.893299408673269</v>
       </c>
-      <c r="C28" s="21" t="n">
+      <c r="C28" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="21" t="n">
+      <c r="D28" s="22" t="n">
         <v>1.317471381777234</v>
       </c>
-      <c r="E28" s="21" t="n">
+      <c r="E28" s="22" t="n">
         <v>4.616413314763465</v>
       </c>
       <c r="F28" s="7" t="n">
@@ -1968,16 +2021,16 @@
           <t>9% p.a. | Direct basket</t>
         </is>
       </c>
-      <c r="B29" s="21" t="n">
+      <c r="B29" s="22" t="n">
         <v>1.876859279147221</v>
       </c>
-      <c r="C29" s="21" t="n">
+      <c r="C29" s="22" t="n">
         <v>0.3607279667886384</v>
       </c>
-      <c r="D29" s="21" t="n">
+      <c r="D29" s="22" t="n">
         <v>1.357871976368822</v>
       </c>
-      <c r="E29" s="21" t="n">
+      <c r="E29" s="22" t="n">
         <v>5.076628806904743</v>
       </c>
       <c r="F29" s="7" t="n">
@@ -2022,7 +2075,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unit 15 risk section: VaR/ES, stress, sizing</t>
+          <t>Sleeve A (growth note) risk: VaR/ES, stress, sizing</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2105,7 @@
           <t>DV01: note change per +1bp rates</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="23" t="n">
         <v>0.0001645165570305362</v>
       </c>
     </row>
@@ -2093,7 +2146,7 @@
           <t>Family net worth (USD)</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="24" t="n">
         <v>2000000000</v>
       </c>
     </row>
@@ -2365,34 +2418,34 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>2330 TT</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>TSMC</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>Foundry / AI accelerators</t>
         </is>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="27" t="n">
         <v>950000</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="27" t="n">
         <v>4000</v>
       </c>
       <c r="H5" s="17">
@@ -2401,384 +2454,384 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>2454 TT</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="25" t="inlineStr">
         <is>
           <t>MediaTek</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="25" t="inlineStr">
         <is>
           <t>Custom AI ASICs / edge AI</t>
         </is>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F6" s="25" t="n"/>
-      <c r="G6" s="25" t="n"/>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
       <c r="H6" s="17">
         <f>IF(OR(F6="",G6=""),"fill",IF(AND(F6&gt;=250,G6&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>000660 KS</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>SK Hynix</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>KR</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>HBM memory</t>
         </is>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F7" s="25" t="n"/>
-      <c r="G7" s="25" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" s="17">
         <f>IF(OR(F7="",G7=""),"fill",IF(AND(F7&gt;=250,G7&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>005930 KS</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="25" t="inlineStr">
         <is>
           <t>Samsung Electronics</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>KR</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="25" t="inlineStr">
         <is>
           <t>HBM / memory</t>
         </is>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F8" s="25" t="n"/>
-      <c r="G8" s="25" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
       <c r="H8" s="17">
         <f>IF(OR(F8="",G8=""),"fill",IF(AND(F8&gt;=250,G8&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>8035 JT</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>Tokyo Electron</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>Wafer-fab equipment</t>
         </is>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F9" s="25" t="n"/>
-      <c r="G9" s="25" t="n"/>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
       <c r="H9" s="17">
         <f>IF(OR(F9="",G9=""),"fill",IF(AND(F9&gt;=250,G9&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="25" t="inlineStr">
         <is>
           <t>6857 JT</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="25" t="inlineStr">
         <is>
           <t>Advantest</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="25" t="inlineStr">
         <is>
           <t>AI chip testing</t>
         </is>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F10" s="25" t="n"/>
-      <c r="G10" s="25" t="n"/>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
       <c r="H10" s="17">
         <f>IF(OR(F10="",G10=""),"fill",IF(AND(F10&gt;=250,G10&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>6146 JT</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>Disco</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="25" t="inlineStr">
         <is>
           <t>Dicing / grinding for HBM</t>
         </is>
       </c>
-      <c r="E11" s="24">
+      <c r="E11" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F11" s="25" t="n"/>
-      <c r="G11" s="25" t="n"/>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
       <c r="H11" s="17">
         <f>IF(OR(F11="",G11=""),"fill",IF(AND(F11&gt;=250,G11&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="25" t="inlineStr">
         <is>
           <t>4063 JT</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>Shin-Etsu Chemical</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="25" t="inlineStr">
         <is>
           <t>Silicon wafers / materials</t>
         </is>
       </c>
-      <c r="E12" s="24">
+      <c r="E12" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F12" s="25" t="n"/>
-      <c r="G12" s="25" t="n"/>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
       <c r="H12" s="17">
         <f>IF(OR(F12="",G12=""),"fill",IF(AND(F12&gt;=250,G12&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>3711 TT</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="25" t="inlineStr">
         <is>
           <t>ASE Technology</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>Advanced packaging</t>
         </is>
       </c>
-      <c r="E13" s="24">
+      <c r="E13" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F13" s="25" t="n"/>
-      <c r="G13" s="25" t="n"/>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
       <c r="H13" s="17">
         <f>IF(OR(F13="",G13=""),"fill",IF(AND(F13&gt;=250,G13&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>4062 JT</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="25" t="inlineStr">
         <is>
           <t>Ibiden</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>JP</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="25" t="inlineStr">
         <is>
           <t>AI chip substrates</t>
         </is>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F14" s="25" t="n"/>
-      <c r="G14" s="25" t="n"/>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
       <c r="H14" s="17">
         <f>IF(OR(F14="",G14=""),"fill",IF(AND(F14&gt;=250,G14&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="25" t="inlineStr">
         <is>
           <t>2317 TT</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Hon Hai (Foxconn)</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D15" s="25" t="inlineStr">
         <is>
           <t>AI server assembly</t>
         </is>
       </c>
-      <c r="E15" s="24">
+      <c r="E15" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F15" s="25" t="n"/>
-      <c r="G15" s="25" t="n"/>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
       <c r="H15" s="17">
         <f>IF(OR(F15="",G15=""),"fill",IF(AND(F15&gt;=250,G15&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>2382 TT</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Quanta Computer</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t>AI servers</t>
         </is>
       </c>
-      <c r="E16" s="24">
+      <c r="E16" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F16" s="25" t="n"/>
-      <c r="G16" s="25" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" s="17">
         <f>IF(OR(F16="",G16=""),"fill",IF(AND(F16&gt;=250,G16&gt;=5),"OK","FAIL"))</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>2308 TT</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Delta Electronics</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="25" t="inlineStr">
         <is>
           <t>Data-centre power / cooling</t>
         </is>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="26">
         <f>1/COUNTA($A$5:$A$17)</f>
         <v/>
       </c>
-      <c r="F17" s="25" t="n"/>
-      <c r="G17" s="25" t="n"/>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
       <c r="H17" s="17">
         <f>IF(OR(F17="",G17=""),"fill",IF(AND(F17&gt;=250,G17&gt;=5),"OK","FAIL"))</f>
         <v/>
@@ -2790,7 +2843,7 @@
           <t>Total weight</t>
         </is>
       </c>
-      <c r="E18" s="24">
+      <c r="E18" s="26">
         <f>SUM(E5:E17)</f>
         <v/>
       </c>
@@ -2823,7 +2876,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Indicative term sheet (links to Pricer)</t>
+          <t>Sleeve A: Asia Digital Bridge growth note (links to Pricer)</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2886,7 @@
           <t>Issuer</t>
         </is>
       </c>
-      <c r="B3" s="26" t="inlineStr">
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>Natixis (guaranteed by BPCE)</t>
         </is>
@@ -2845,7 +2898,7 @@
           <t>Client</t>
         </is>
       </c>
-      <c r="B4" s="26" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>NKE Private Wealth (Chak family office)</t>
         </is>
@@ -2857,7 +2910,7 @@
           <t>Notional</t>
         </is>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="29">
         <f>TEXT(Pricer!B5,"$#,##0")</f>
         <v/>
       </c>
@@ -2868,7 +2921,7 @@
           <t>Currency</t>
         </is>
       </c>
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>USD; underlying quanto (no FX exposure)</t>
         </is>
@@ -2880,7 +2933,7 @@
           <t>Trade / issue date</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="28" t="inlineStr">
         <is>
           <t>17 Sep 2026</t>
         </is>
@@ -2892,7 +2945,7 @@
           <t>Maturity</t>
         </is>
       </c>
-      <c r="B8" s="27">
+      <c r="B8" s="29">
         <f>"Sep "&amp;(2026+Pricer!B6)&amp;" ("&amp;Pricer!B6&amp;"Y)"</f>
         <v/>
       </c>
@@ -2903,7 +2956,7 @@
           <t>Underlying</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="28" t="inlineStr">
         <is>
           <t>Natixis Asia Digital Bridge 10% VT Index (USD, 1% decrement), on an equal-weight basket of 13 Asian AI-hardware stocks</t>
         </is>
@@ -2915,7 +2968,7 @@
           <t>Index rules</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Daily exposure = min(10% / max(20d, 60d realised vol), 150%), cash on the remainder, minus 1% p.a.</t>
         </is>
@@ -2927,7 +2980,7 @@
           <t>Capital protection</t>
         </is>
       </c>
-      <c r="B11" s="27">
+      <c r="B11" s="29">
         <f>TEXT(Pricer!B7,"0%")&amp;" at maturity, subject to issuer credit"</f>
         <v/>
       </c>
@@ -2938,8 +2991,8 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B12" s="27">
-        <f>TEXT(Pricer!B23,"0%")&amp;" of index performance, uncapped"</f>
+      <c r="B12" s="29">
+        <f>TEXT(Pricer!B29,"0%")&amp;" of index performance, uncapped (with Legacy Lock and 12M averaging)"</f>
         <v/>
       </c>
     </row>
@@ -2949,21 +3002,21 @@
           <t>Redemption</t>
         </is>
       </c>
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Protection + Participation x max(0, Index final / Index initial - 1)</t>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>Protection + Participation x max(0, average final index perf, locked gain)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Optional enhancements</t>
-        </is>
-      </c>
-      <c r="B14" s="26" t="inlineStr">
-        <is>
-          <t>12M final averaging (raises participation); Legacy Lock 130/160/190 (lowers it); see MC Results</t>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>12M final averaging; Legacy Lock floors gains at +30/+60/+90% once hit on an annual date</t>
         </is>
       </c>
     </row>
@@ -2973,7 +3026,7 @@
           <t>Appendix variant</t>
         </is>
       </c>
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>Best-of with a spot Bitcoin ETF sleeve (IBIT US); not in the core proposal</t>
         </is>
@@ -2985,7 +3038,7 @@
           <t>Secondary market</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Natixis indicative daily bid, under normal market conditions</t>
         </is>
@@ -2997,7 +3050,7 @@
           <t>Pricing basis</t>
         </is>
       </c>
-      <c r="B17" s="26" t="inlineStr">
+      <c r="B17" s="28" t="inlineStr">
         <is>
           <t>Funding from the game-rules grid; option inputs are placeholders to be refreshed on Bloomberg</t>
         </is>
@@ -3006,4 +3059,970 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sleeve B: AI Hardware Phoenix, 10% p.a. conditional coupon autocall (USD, 5Y)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Blue = input, black = formula, green = link. MC outputs pasted from pricing/scenario2_barbell.py (placeholder market inputs).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Terms</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>P(called by end of year)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Probability</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Notional (USD)</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>Barbell!B4*Barbell!B6</f>
+        <v/>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>0.705975</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Tenor (years)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0.79675</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Coupon p.a. (paid quarterly)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>0.838575</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Coupon barrier (basket vs initial)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0.862075</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Autocall trigger, year 1</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>0.875575</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Autocall step-down per year</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Capital barrier at maturity (European)</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Capital barrier menu</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Natixis margin</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>P(loss)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Underlying</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Equal-weight basket: TSMC (2330 TT), SK Hynix (000660 KS), Tokyo Electron (8035 JT); USD quanto</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>0.01241396916887405</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>0.06934999999999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Quarterly coupon</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>B7/4</f>
+        <v/>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.02260196363677791</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>0.09365</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="D14" s="8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.02821602704729953</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0.1101</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Monte Carlo outputs</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>0.0310840170827098</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0.1208</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Fair value (% notional, discounted at Natixis funding)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.9782719301521816</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Natixis margin</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.02172806984781839</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Stress (spot and vol together)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Phoenix MTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Expected life (years)</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="n">
+        <v>1.27523125</v>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>AI hardware crash: stocks -30%, vol x1.5</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>0.7430077777709048</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Expected coupons paid (% notional)</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.09715749999999991</v>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>Taiwan gap: stocks -20%, vol x1.3</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>0.841857169089921</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>P(capital loss)</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.090375</v>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>Rates +100bp</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>0.9683534008840489</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Expected loss (% notional)</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.06217147939324468</v>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Rally: stocks +20%</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>1.005464476360348</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>PV of coupons</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.08990802287804203</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>PV of principal repaid at par</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>0.93550739535112</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>PV of short put (barrier loss)</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>0.04714348807698036</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Check: coupons + principal - put = fair value</t>
+        </is>
+      </c>
+      <c r="B25" s="17">
+        <f>IF(ABS(B22+B23-B24-B16)&lt;0.0005,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Scenario cash flows (% notional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Quarters of coupon</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Basket at end</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Redemption</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Total cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Called at Q1 (basket &gt;= 100%)</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="11">
+        <f>IF(D29&lt;$B$11,D29,1)</f>
+        <v/>
+      </c>
+      <c r="F29" s="11">
+        <f>E29+B29*$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Called in year 2 (basket at 96% vs 95% trigger)</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E30" s="11">
+        <f>IF(D30&lt;$B$11,D30,1)</f>
+        <v/>
+      </c>
+      <c r="F30" s="11">
+        <f>E30+B30*$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Never called, basket 70% at maturity, all coupons paid</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E31" s="11">
+        <f>IF(D31&lt;$B$11,D31,1)</f>
+        <v/>
+      </c>
+      <c r="F31" s="11">
+        <f>E31+B31*$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Basket 45% at maturity, coupons stop after year 2</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E32" s="11">
+        <f>IF(D32&lt;$B$11,D32,1)</f>
+        <v/>
+      </c>
+      <c r="F32" s="11">
+        <f>E32+B32*$B$13</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Barbell allocation: protect with Sleeve A, earn income with Sleeve B</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Edit the blue cells. Simulated outcomes are pasted from pricing/scenario2_barbell.py (forward simulation, not a backtest).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Total mandate (USD)</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Sleeve A: growth note allocation</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Sleeve B: Phoenix allocation</t>
+        </is>
+      </c>
+      <c r="B6" s="13">
+        <f>1-B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Sleeve A amount (USD)</t>
+        </is>
+      </c>
+      <c r="B7" s="16">
+        <f>B4*B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Sleeve B amount (USD)</t>
+        </is>
+      </c>
+      <c r="B8" s="16">
+        <f>B4*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Capital protected at maturity (USD, ex issuer default)</t>
+        </is>
+      </c>
+      <c r="B9" s="16">
+        <f>B7*Pricer!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Contractual worst case (Phoenix basket to zero, before coupons)</t>
+        </is>
+      </c>
+      <c r="B10" s="13">
+        <f>B9/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Phoenix coupon income per year if paid (USD)</t>
+        </is>
+      </c>
+      <c r="B11" s="16">
+        <f>B8*Phoenix!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>Family net worth (USD)</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>2000000000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Contractual worst-case loss as % of net worth</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>(B4-B9)/B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>7Y outcome (multiple of capital)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>5th pct</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Median</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>95th pct</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>P(&lt;100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>3% basket return | Barbell 60/40</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="n">
+        <v>0.8351458043525511</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>1.265140019113114</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>1.3156006157922</v>
+      </c>
+      <c r="E16" s="22" t="n">
+        <v>1.799087910112445</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>0.08683333333333333</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>3% basket return | Growth note only</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="22" t="n">
+        <v>1.199488444220527</v>
+      </c>
+      <c r="D17" s="22" t="n">
+        <v>1.335947433776066</v>
+      </c>
+      <c r="E17" s="22" t="n">
+        <v>2.101480293168121</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>3% basket return | Phoenix only (cash to 7Y)</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="n">
+        <v>0.5602206860000741</v>
+      </c>
+      <c r="C18" s="22" t="n">
+        <v>1.314145876690479</v>
+      </c>
+      <c r="D18" s="22" t="n">
+        <v>1.285080388816403</v>
+      </c>
+      <c r="E18" s="22" t="n">
+        <v>1.559656446123209</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0.0925</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>3% basket return | Direct basket</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="n">
+        <v>0.2155872178156426</v>
+      </c>
+      <c r="C19" s="22" t="n">
+        <v>0.8140358498142535</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <v>1.117407904135875</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <v>3.041919006768048</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.5998333333333333</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>6% basket return | Barbell 60/40</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n">
+        <v>0.9029327705481972</v>
+      </c>
+      <c r="C20" s="22" t="n">
+        <v>1.35490321595094</v>
+      </c>
+      <c r="D20" s="22" t="n">
+        <v>1.384030925097693</v>
+      </c>
+      <c r="E20" s="22" t="n">
+        <v>1.922449999537918</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0.06358333333333334</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>6% basket return | Growth note only</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="22" t="n">
+        <v>1.345291788578202</v>
+      </c>
+      <c r="D21" s="22" t="n">
+        <v>1.438312646702159</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>2.300983325737862</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>6% basket return | Phoenix only (cash to 7Y)</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="n">
+        <v>0.6903658228966442</v>
+      </c>
+      <c r="C22" s="22" t="n">
+        <v>1.314145876690479</v>
+      </c>
+      <c r="D22" s="22" t="n">
+        <v>1.302608342690993</v>
+      </c>
+      <c r="E22" s="22" t="n">
+        <v>1.560214404815371</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0.06966666666666667</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>6% basket return | Direct basket</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="n">
+        <v>0.268760531146695</v>
+      </c>
+      <c r="C23" s="22" t="n">
+        <v>0.9883675610719496</v>
+      </c>
+      <c r="D23" s="22" t="n">
+        <v>1.375361289893981</v>
+      </c>
+      <c r="E23" s="22" t="n">
+        <v>3.707936692022572</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0.50625</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>9% basket return | Barbell 60/40</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="n">
+        <v>1.125658350676192</v>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>1.428760027017175</v>
+      </c>
+      <c r="D24" s="22" t="n">
+        <v>1.459194645090567</v>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>2.027582648519454</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>0.04066666666666666</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>9% basket return | Growth note only</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>1.499692028764449</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <v>1.551278032529135</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <v>2.499076086293346</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>9% basket return | Phoenix only (cash to 7Y)</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="n">
+        <v>1.201305525553019</v>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>1.314145876690479</v>
+      </c>
+      <c r="D26" s="22" t="n">
+        <v>1.321069563932717</v>
+      </c>
+      <c r="E26" s="22" t="n">
+        <v>1.559692028247597</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>0.04758333333333333</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>9% basket return | Direct basket</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="n">
+        <v>0.3335538986024838</v>
+      </c>
+      <c r="C27" s="22" t="n">
+        <v>1.239572979110937</v>
+      </c>
+      <c r="D27" s="22" t="n">
+        <v>1.691036671964204</v>
+      </c>
+      <c r="E27" s="22" t="n">
+        <v>4.435428579625211</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>0.3901666666666667</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Phoenix cash (coupons, early redemption) is assumed reinvested at USD cash 3.75% until year 7; rolling into a new Phoenix would raise the barbell's income.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>